<commit_message>
feat(inspecciones-internas): UI dark mode, Excel solid colors fix, Grouped Levantamiento emails
</commit_message>
<xml_diff>
--- a/public/templates/digital/Inspecciones Internas SSOMA.xlsx
+++ b/public/templates/digital/Inspecciones Internas SSOMA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlcan\Desktop\Seguimiento de plataforma de seguridad Antigravity\ssoma-platform\public\templates\digital\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85FE2CD-E978-4057-946A-ED7C39E2B6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3FDC3B-97F7-4CCD-B222-55EFD489DDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -174,7 +174,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="94">
   <si>
     <t>INSPECCIONES INTERNAS DE SEGURIDAD, SALUD EN EL TRABAJO Y MEDIO AMBIENTE</t>
   </si>
@@ -459,6 +459,9 @@
   </si>
   <si>
     <t>MEDIO AMBIENTE</t>
+  </si>
+  <si>
+    <t>EVIDENCIA DE LEVANTAMIENTO</t>
   </si>
 </sst>
 </file>
@@ -1433,7 +1436,75 @@
     <cellStyle name="Título 3" xfId="39" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="40" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="0"/>
@@ -2986,7 +3057,9 @@
       <c r="P14" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="Q14" s="24"/>
+      <c r="Q14" s="24" t="s">
+        <v>93</v>
+      </c>
       <c r="R14" s="24"/>
       <c r="S14" s="24"/>
       <c r="T14" s="24"/>
@@ -3375,30 +3448,6 @@
     <mergeCell ref="P4:S4"/>
     <mergeCell ref="T4:U4"/>
   </mergeCells>
-  <conditionalFormatting sqref="J3 J8:J1048576">
-    <cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="RIESGO ALTO">
-      <formula>NOT(ISERROR(SEARCH("RIESGO ALTO",J3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="RIESGO MEDIO">
-      <formula>NOT(ISERROR(SEARCH("RIESGO MEDIO",J3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="RIESGO BAJO">
-      <formula>NOT(ISERROR(SEARCH("RIESGO BAJO",J3)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K15:K21">
-    <cfRule type="expression" dxfId="8" priority="6">
-      <formula>"RIESGO BAJO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U15:U21">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
-      <formula>"Cerrado"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
-      <formula>"Abierto"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.39370078740157483" header="0" footer="0.19685039370078741"/>
   <pageSetup paperSize="9" scale="47" fitToHeight="3" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -4199,26 +4248,26 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="J3 J8:J1048576">
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="RIESGO ALTO">
+    <cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="RIESGO ALTO">
       <formula>NOT(ISERROR(SEARCH("RIESGO ALTO",J3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="RIESGO MEDIO">
+    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="RIESGO MEDIO">
       <formula>NOT(ISERROR(SEARCH("RIESGO MEDIO",J3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="RIESGO BAJO">
+    <cfRule type="containsText" dxfId="9" priority="6" operator="containsText" text="RIESGO BAJO">
       <formula>NOT(ISERROR(SEARCH("RIESGO BAJO",J3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K15:K18">
-    <cfRule type="expression" dxfId="2" priority="10">
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>"RIESGO BAJO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U15:U18">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"Cerrado"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>"Abierto"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4529,6 +4578,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2b230e36-0a53-4ac0-ac01-c22c1efbb34c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e841f38b-9f23-43dc-9de2-cda5176cd52a" xsi:nil="true"/>
+    <SharedWithUsers xmlns="e841f38b-9f23-43dc-9de2-cda5176cd52a">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101002CDB6831020C52409B02D6F92027612F" ma:contentTypeVersion="19" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="8a6c93356d472a3cd4cd316c29954489">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2b230e36-0a53-4ac0-ac01-c22c1efbb34c" xmlns:ns3="e841f38b-9f23-43dc-9de2-cda5176cd52a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="282de175f270af219a6e0391fb3ffa13" ns2:_="" ns3:_="">
     <xsd:import namespace="2b230e36-0a53-4ac0-ac01-c22c1efbb34c"/>
@@ -4789,34 +4865,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2b230e36-0a53-4ac0-ac01-c22c1efbb34c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e841f38b-9f23-43dc-9de2-cda5176cd52a" xsi:nil="true"/>
-    <SharedWithUsers xmlns="e841f38b-9f23-43dc-9de2-cda5176cd52a">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C40FEBFB-4C1D-42B9-BBE1-4206E3FA25E5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2b230e36-0a53-4ac0-ac01-c22c1efbb34c"/>
+    <ds:schemaRef ds:uri="e841f38b-9f23-43dc-9de2-cda5176cd52a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32903455-E3DE-4AD9-97CB-8F70F1C84E4E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05392383-55EC-41F2-B63B-3F43488FA23A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4833,23 +4901,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C40FEBFB-4C1D-42B9-BBE1-4206E3FA25E5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2b230e36-0a53-4ac0-ac01-c22c1efbb34c"/>
-    <ds:schemaRef ds:uri="e841f38b-9f23-43dc-9de2-cda5176cd52a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32903455-E3DE-4AD9-97CB-8F70F1C84E4E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>